<commit_message>
crypto-dex-perp: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -2141,9 +2141,9 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Open the trading screen, select ETH/USD through the pair dropdown, wait for the 24H VOLUME figure
-Read the header price by label; GET prices/tickers
-Expect |screen - ticker| / ticker &lt;= 0.5%</t>
+          <t>1. Open the trading screen, select ETH/USD through the pair dropdown, wait for the 24H VOLUME figure
+2. Read the header price by label; GET prices/tickers
+3. Expect |screen - ticker| / ticker &lt;= 0.5%</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -2193,9 +2193,9 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Open the trading screen, select BTC/USD through the pair dropdown, wait for the 24H VOLUME figure
-Read the header price by label; GET prices/tickers
-Expect |screen - ticker| / ticker &lt;= 0.5%</t>
+          <t>1. Open the trading screen, select BTC/USD through the pair dropdown, wait for the 24H VOLUME figure
+2. Read the header price by label; GET prices/tickers
+3. Expect |screen - ticker| / ticker &lt;= 0.5%</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2245,9 +2245,9 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Open the trading screen, select SOL/USD through the pair dropdown, wait for the 24H VOLUME figure
-Read the header price by label; GET prices/tickers
-Expect |screen - ticker| / ticker &lt;= 0.5%</t>
+          <t>1. Open the trading screen, select SOL/USD through the pair dropdown, wait for the 24H VOLUME figure
+2. Read the header price by label; GET prices/tickers
+3. Expect |screen - ticker| / ticker &lt;= 0.5%</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2297,9 +2297,9 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Read OPEN INTEREST long and short off the header, with the rounding unit shown
-GET v1/markets/values (interestInTokens) and prices/tickers (price)
-Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
+          <t>1. Read OPEN INTEREST long and short off the header, with the rounding unit shown
+2. GET v1/markets/values (interestInTokens) and prices/tickers (price)
+3. Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -2349,9 +2349,9 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Read OPEN INTEREST long and short off the header, with the rounding unit shown
-GET v1/markets/values (interestInTokens) and prices/tickers (price)
-Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
+          <t>1. Read OPEN INTEREST long and short off the header, with the rounding unit shown
+2. GET v1/markets/values (interestInTokens) and prices/tickers (price)
+3. Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2401,9 +2401,9 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Read OPEN INTEREST long and short off the header, with the rounding unit shown
-GET v1/markets/values (interestInTokens) and prices/tickers (price)
-Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
+          <t>1. Read OPEN INTEREST long and short off the header, with the rounding unit shown
+2. GET v1/markets/values (interestInTokens) and prices/tickers (price)
+3. Expect |screen - tokens x price| &lt;= display unit + 2% of the value (prices move between reads)</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2453,8 +2453,8 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Read the (L%/S%) split and the two OI amounts from the same header line
-Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
+          <t>1. Read the (L%/S%) split and the two OI amounts from the same header line
+2. Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2504,8 +2504,8 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Read the (L%/S%) split and the two OI amounts from the same header line
-Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
+          <t>1. Read the (L%/S%) split and the two OI amounts from the same header line
+2. Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2555,8 +2555,8 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Read the (L%/S%) split and the two OI amounts from the same header line
-Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
+          <t>1. Read the (L%/S%) split and the two OI amounts from the same header line
+2. Expect L% within 1 point of long / (long + short) x 100, allowing for the rounding of both</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2606,8 +2606,8 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Read the header price; eth_call Vault.getMaxPrice(WETH) on Arbitrum, scale by 1e30
-Expect |screen - chain| / chain &lt;= 0.5%</t>
+          <t>1. Read the header price; eth_call Vault.getMaxPrice(WETH) on Arbitrum, scale by 1e30
+2. Expect |screen - chain| / chain &lt;= 0.5%</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -2657,8 +2657,8 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Read the header price; eth_call Vault.getMaxPrice(WBTC) on Arbitrum, scale by 1e30
-Expect |screen - chain| / chain &lt;= 0.5%</t>
+          <t>1. Read the header price; eth_call Vault.getMaxPrice(WBTC) on Arbitrum, scale by 1e30
+2. Expect |screen - chain| / chain &lt;= 0.5%</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">

</xml_diff>